<commit_message>
Sheets: batteries written out in full (72 men, 8 guns) with gun names
Artillery rows name their guns (old smoothbore / smoothbore / rifled /
breech-loading guns) instead of musket names; a standard battery is
exported as its real crew and guns instead of blank cells.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/players/battle_template.xlsx
+++ b/players/battle_template.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -491,50 +491,57 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  "Should it break?": yes, no, or blank if you have no view.</t>
+          <t xml:space="preserve">  Weapon: muskets for infantry and cavalry; for artillery, the guns (smoothbore guns, rifled guns, ...).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Orders tab: what each unit does, round by round. A round is a stretch of time (e.g. 60 or 90 minutes).</t>
+          <t xml:space="preserve">  "Should it break?": yes, no, or blank if you have no view.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  fire = shoot at the Target; charge = close and fight hand to hand; hold = stay put. Units without a row hold.</t>
+          <t>Orders tab: what each unit does, round by round. A round is a stretch of time (e.g. 60 or 90 minutes).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Artillery can pick Ammo: round shot (long range), shell, or canister (close range).</t>
+          <t xml:space="preserve">  fire = shoot at the Target; charge = close and fight hand to hand; hold = stay put. Units without a row hold.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Not sure how to write the orders? Describe the plan in Notes on the Battle tab and we will write them.</t>
+          <t xml:space="preserve">  Artillery can pick Ammo: round shot (long range), shell, or canister (close range).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Not sure how to write the orders? Describe the plan in Notes on the Battle tab and we will write them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Feedback tab: after you have seen the engine's report, rate how it felt. Copy the engine version from the report.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>How to send it back: Google Sheets: File &gt; Download &gt; Microsoft Excel (.xlsx). Excel: just save. Send us the file.</t>
         </is>
@@ -839,7 +846,7 @@
       <formula1>"irregulars,light,line,marine,pikes,dragoons,heavy,battery,horse battery,siege battery"</formula1>
     </dataValidation>
     <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"unarmed / pikes,matchlock,smoothbore musket,rifled musket,needle rifle"</formula1>
+      <formula1>"unarmed / pikes,matchlock,smoothbore musket,rifled musket,needle rifle,old smoothbore guns,smoothbore guns,rifled guns,breech-loading guns"</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"yes,no"</formula1>

</xml_diff>